<commit_message>
Update the case studies with review fixes
Corrected notes for Saltbrush and Sunfield, two decimal backlog coverage for Aldercrest, and rebuilt workbooks.
</commit_message>
<xml_diff>
--- a/aldercrest-aerospace/Aldercrest_FY2025_Financial_Model.xlsx
+++ b/aldercrest-aerospace/Aldercrest_FY2025_Financial_Model.xlsx
@@ -668,13 +668,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0_);(#,##0);&quot;-&quot;_)"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.00%"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="#,##0"/>
     <numFmt numFmtId="168" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="0.00"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -865,9 +866,9 @@
     </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="168" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>

</xml_diff>